<commit_message>
adicionadas as fotos do café trindade no ficheiro aux
</commit_message>
<xml_diff>
--- a/DRIVE/3. Operações/3.1 Projetos/26003 - CAFE TRINDADE 1961 (São João da Madeira)/Peças escritas/PRÉ-ORÇAMENTO HB V1 SAO-2026-0003-ESPL.xlsx
+++ b/DRIVE/3. Operações/3.1 Projetos/26003 - CAFE TRINDADE 1961 (São João da Madeira)/Peças escritas/PRÉ-ORÇAMENTO HB V1 SAO-2026-0003-ESPL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\castr\MINDSET\DRIVE\3. Operações\3.1 Projetos\26003 - CAFE TRINDADE 1961 (São João da Madeira)\Peças escritas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruisa\mindset\MINDSET\DRIVE\3. Operações\3.1 Projetos\26003 - CAFE TRINDADE 1961 (São João da Madeira)\Peças escritas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07BB4C00-8696-4823-B56F-97661E5D952D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92228E51-3938-41F0-B96C-72E122A9A366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proposta" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
imprimir orçamentos cafe trindade
</commit_message>
<xml_diff>
--- a/DRIVE/3. Operações/3.1 Projetos/26003 - CAFE TRINDADE 1961 (São João da Madeira)/Peças escritas/PRÉ-ORÇAMENTO HB V1 SAO-2026-0003-ESPL.xlsx
+++ b/DRIVE/3. Operações/3.1 Projetos/26003 - CAFE TRINDADE 1961 (São João da Madeira)/Peças escritas/PRÉ-ORÇAMENTO HB V1 SAO-2026-0003-ESPL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\castr\MINDSET\DRIVE\3. Operações\3.1 Projetos\26003 - CAFE TRINDADE 1961 (São João da Madeira)\Peças escritas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{406FC34E-93A8-46F0-861F-09FCF8A04E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B04ED7A0-8EF8-4936-8C79-2714C256743A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Proposta" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Proposta!$A$1:$G$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Proposta!$A$1:$G$63</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -37,10 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
-  <si>
-    <t>PROPOSTA DE FORNECIMENTO</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>A confirmar</t>
   </si>
@@ -114,25 +111,37 @@
     <t>Cabo paralelo bobine — 100m</t>
   </si>
   <si>
-    <t>Mao de obra especializada</t>
-  </si>
-  <si>
     <t xml:space="preserve">Café Trindade 1961 </t>
   </si>
   <si>
-    <t>30 dias</t>
-  </si>
-  <si>
-    <t>Pré-Pagamento</t>
-  </si>
-  <si>
     <t>Audibax Pro Fiji 6  (Par)</t>
   </si>
   <si>
-    <t>Coluna passiva 6" 2 Vías 50W RMS c/ suporte de parede IP65 (preto e branco)</t>
-  </si>
-  <si>
     <t>NOTAS: Deslocações a decidir. Preços por unidade apresentados não incluem IVA.Orçamento sujeito a revisões.</t>
+  </si>
+  <si>
+    <t>Até aprovação do cliente</t>
+  </si>
+  <si>
+    <t>Pago na encomenda</t>
+  </si>
+  <si>
+    <t>PROPOSTA DE FORNECIMENTO (MAIS CARO)</t>
+  </si>
+  <si>
+    <t>Tubo VD20</t>
+  </si>
+  <si>
+    <t>Tubo rigido c/ acessórios</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Mao de obra especializada, prazo de entrega: 1 dia.</t>
+  </si>
+  <si>
+    <t>Coluna passiva 15cm 2 Vías 50W RMS c/ suporte de parede e IP65 (preto ou branco)</t>
   </si>
 </sst>
 </file>
@@ -143,7 +152,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00&quot; €&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -192,6 +201,69 @@
     </font>
     <font>
       <b/>
+      <sz val="8"/>
+      <color rgb="FF888888"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="0" tint="-0.34998626667073579"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF1A1A1A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="7"/>
+      <color rgb="FF888888"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FFE8B800"/>
       <name val="Arial"/>
@@ -206,64 +278,14 @@
     </font>
     <font>
       <b/>
-      <sz val="8"/>
-      <color rgb="FF888888"/>
+      <sz val="9"/>
+      <color rgb="FF1A1A1A"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <i/>
-      <sz val="8"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="9"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color theme="0" tint="-0.34998626667073579"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
-      <color rgb="FF1A1A1A"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="7"/>
-      <color rgb="FF888888"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -474,7 +496,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -492,42 +514,36 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="4" fontId="4" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="15" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="15" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
@@ -540,7 +556,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -549,13 +565,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -563,44 +579,62 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -723,7 +757,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="66265" y="1"/>
-          <a:ext cx="861132" cy="858329"/>
+          <a:ext cx="862166" cy="852812"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -917,101 +951,101 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="15.77734375" customWidth="1"/>
     <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="19.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" customWidth="1"/>
     <col min="7" max="7" width="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:7" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36"/>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="F2" s="55"/>
-      <c r="G2" s="39"/>
-    </row>
-    <row r="3" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:9" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="34"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="61" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="61"/>
+      <c r="G2" s="37"/>
+    </row>
+    <row r="3" spans="1:9" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="14"/>
+      <c r="E4" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1"/>
+      <c r="B5" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="17" t="s">
+      <c r="C5" s="17">
+        <v>46152</v>
+      </c>
+      <c r="D5" s="18"/>
+      <c r="E5" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
-      <c r="B5" s="18" t="s">
+      <c r="F5" s="20"/>
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="19">
-        <v>46147</v>
-      </c>
-      <c r="D5" s="20"/>
-      <c r="E5" s="21" t="s">
+      <c r="C6" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="18"/>
+      <c r="E6" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="22"/>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1"/>
-      <c r="B6" s="18" t="s">
+      <c r="F6" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="23"/>
+      <c r="B7" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="20"/>
-      <c r="E6" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="25"/>
-      <c r="B7" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="D7" s="20"/>
-      <c r="E7" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="24" t="s">
+      <c r="C7" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" s="18"/>
+      <c r="E7" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="26"/>
-    </row>
-    <row r="8" spans="1:7" ht="3.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F7" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="24"/>
+    </row>
+    <row r="8" spans="1:9" ht="3.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1020,37 +1054,37 @@
       <c r="F8" s="4"/>
       <c r="G8" s="5"/>
     </row>
-    <row r="9" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="27"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="29"/>
-    </row>
-    <row r="10" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="25"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="27"/>
+    </row>
+    <row r="10" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="41" t="s">
+      <c r="B10" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="39" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="42" t="s">
+      <c r="E10" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="E10" s="43" t="s">
+      <c r="F10" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="F10" s="43" t="s">
-        <v>5</v>
-      </c>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="60">
+      <c r="B11" s="59">
         <v>2</v>
       </c>
       <c r="C11" s="9"/>
@@ -1059,11 +1093,11 @@
       <c r="F11" s="9"/>
       <c r="G11" s="10"/>
     </row>
-    <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="60"/>
+      <c r="B12" s="59"/>
       <c r="C12" s="6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D12" s="7">
         <f>189*1.3</f>
@@ -1073,26 +1107,29 @@
         <f>B11*D12</f>
         <v>491.40000000000003</v>
       </c>
-      <c r="F12" s="13">
+      <c r="F12" s="11">
         <f>E12</f>
         <v>491.40000000000003</v>
       </c>
       <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="54"/>
-      <c r="C13" s="35" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30"/>
+      <c r="B13" s="60"/>
+      <c r="C13" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="53">
+      <c r="B14" s="58">
         <v>1</v>
       </c>
       <c r="C14" s="9"/>
@@ -1101,11 +1138,11 @@
       <c r="F14" s="9"/>
       <c r="G14" s="10"/>
     </row>
-    <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="60"/>
+      <c r="B15" s="59"/>
       <c r="C15" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D15" s="7">
         <f>115*1.3</f>
@@ -1115,26 +1152,26 @@
         <f>B14*D15</f>
         <v>149.5</v>
       </c>
-      <c r="F15" s="13">
+      <c r="F15" s="11">
         <f>E15</f>
         <v>149.5</v>
       </c>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="54"/>
-      <c r="C16" s="35" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
+      <c r="B16" s="60"/>
+      <c r="C16" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
       <c r="G16" s="2"/>
     </row>
     <row r="17" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="53">
+      <c r="B17" s="58">
         <v>1</v>
       </c>
       <c r="C17" s="9"/>
@@ -1145,9 +1182,9 @@
     </row>
     <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="60"/>
+      <c r="B18" s="59"/>
       <c r="C18" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D18" s="7">
         <f>110*1.3</f>
@@ -1157,7 +1194,7 @@
         <f>B17*D18</f>
         <v>143</v>
       </c>
-      <c r="F18" s="13">
+      <c r="F18" s="11">
         <f>E18</f>
         <v>143</v>
       </c>
@@ -1165,18 +1202,18 @@
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="54"/>
-      <c r="C19" s="35" t="s">
-        <v>24</v>
-      </c>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
+      <c r="B19" s="60"/>
+      <c r="C19" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="53">
+      <c r="B20" s="58">
         <v>1</v>
       </c>
       <c r="C20" s="9"/>
@@ -1187,9 +1224,9 @@
     </row>
     <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="60"/>
+      <c r="B21" s="59"/>
       <c r="C21" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D21" s="7">
         <f>180*1.3</f>
@@ -1199,7 +1236,7 @@
         <f>B20*D21</f>
         <v>234</v>
       </c>
-      <c r="F21" s="13">
+      <c r="F21" s="11">
         <f>E21</f>
         <v>234</v>
       </c>
@@ -1207,18 +1244,20 @@
     </row>
     <row r="22" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="B22" s="54"/>
-      <c r="C22" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
+      <c r="B22" s="60"/>
+      <c r="C22" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
       <c r="G22" s="2"/>
     </row>
     <row r="23" spans="1:7" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
-      <c r="B23" s="53"/>
+      <c r="B23" s="58">
+        <v>1</v>
+      </c>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
@@ -1226,98 +1265,126 @@
       <c r="G23" s="10"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="25"/>
-      <c r="B24" s="54"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="31"/>
-    </row>
-    <row r="25" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
+      <c r="B24" s="59"/>
+      <c r="C24" s="56" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24" s="57">
+        <f>61.54*1.3</f>
+        <v>80.001999999999995</v>
+      </c>
+      <c r="E24" s="8">
+        <f>D24*B23</f>
+        <v>80.001999999999995</v>
+      </c>
+      <c r="F24" s="11">
+        <f>E24</f>
+        <v>80.001999999999995</v>
+      </c>
+      <c r="G24" s="2"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
-      <c r="D25" s="11"/>
-      <c r="F25" s="12"/>
+      <c r="B25" s="60"/>
+      <c r="C25" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="D25" s="28"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="G26" s="2"/>
-    </row>
-    <row r="27" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="1"/>
-      <c r="G27" s="2"/>
+      <c r="B26" s="52"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="10"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="23"/>
+      <c r="B27" s="53"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="29"/>
     </row>
     <row r="28" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
+      <c r="D28" s="54"/>
+      <c r="F28" s="55"/>
       <c r="G28" s="2"/>
     </row>
-    <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
-      <c r="F29" s="61"/>
       <c r="G29" s="2"/>
     </row>
     <row r="30" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="G30" s="2"/>
     </row>
-    <row r="31" spans="1:7" ht="3.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="G31" s="2"/>
     </row>
-    <row r="32" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="G32" s="2"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="G33" s="2"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
+      <c r="F34" s="51"/>
       <c r="G34" s="2"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="G35" s="2"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" ht="3.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="G36" s="2"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" ht="3.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="G37" s="2"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" ht="3.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="G38" s="2"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" ht="3.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="G39" s="2"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" ht="3.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="G40" s="2"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" ht="3.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="G41" s="2"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" ht="3.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="G42" s="2"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="G43" s="2"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" ht="67.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="G44" s="2"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="G45" s="2"/>
     </row>
@@ -1325,70 +1392,118 @@
       <c r="A46" s="1"/>
       <c r="G46" s="2"/>
     </row>
-    <row r="47" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A47" s="44"/>
-      <c r="B47" s="45"/>
-      <c r="C47" s="45"/>
-      <c r="D47" s="46" t="s">
-        <v>19</v>
-      </c>
-      <c r="E47" s="46"/>
-      <c r="F47" s="47">
-        <f>F12+F15+F18+F21</f>
-        <v>1017.9000000000001</v>
-      </c>
-      <c r="G47" s="48"/>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="1"/>
+      <c r="G47" s="2"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="G48" s="2"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" s="56" t="s">
-        <v>31</v>
-      </c>
-      <c r="B49" s="57"/>
-      <c r="C49" s="57"/>
-      <c r="D49" s="57"/>
-      <c r="E49" s="57"/>
-      <c r="F49" s="57"/>
-      <c r="G49" s="58"/>
-    </row>
-    <row r="50" spans="1:7" ht="5.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="32"/>
-      <c r="B50" s="33"/>
-      <c r="C50" s="33"/>
-      <c r="D50" s="33"/>
-      <c r="E50" s="33"/>
-      <c r="F50" s="33"/>
-      <c r="G50" s="34"/>
-    </row>
-    <row r="51" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="49"/>
-      <c r="B51" s="50" t="s">
-        <v>7</v>
-      </c>
-      <c r="C51" s="51"/>
-      <c r="D51" s="59" t="s">
-        <v>11</v>
-      </c>
-      <c r="E51" s="59"/>
-      <c r="F51" s="59"/>
-      <c r="G51" s="52"/>
+      <c r="A49" s="1"/>
+      <c r="G49" s="2"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" s="1"/>
+      <c r="G50" s="2"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" s="1"/>
+      <c r="G51" s="2"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" s="1"/>
+      <c r="G52" s="2"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" s="1"/>
+      <c r="G53" s="2"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" s="1"/>
+      <c r="G54" s="2"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" s="1"/>
+      <c r="G55" s="2"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" s="1"/>
+      <c r="G56" s="2"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" s="1"/>
+      <c r="G57" s="2"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" s="1"/>
+      <c r="G58" s="2"/>
+    </row>
+    <row r="59" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A59" s="42"/>
+      <c r="B59" s="43"/>
+      <c r="C59" s="43"/>
+      <c r="D59" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="E59" s="44"/>
+      <c r="F59" s="45">
+        <f>F12+F15+F18+F21+F24</f>
+        <v>1097.902</v>
+      </c>
+      <c r="G59" s="46"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" s="1"/>
+      <c r="G60" s="2"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61" s="62" t="s">
+        <v>26</v>
+      </c>
+      <c r="B61" s="63"/>
+      <c r="C61" s="63"/>
+      <c r="D61" s="63"/>
+      <c r="E61" s="63"/>
+      <c r="F61" s="63"/>
+      <c r="G61" s="64"/>
+    </row>
+    <row r="62" spans="1:7" ht="5.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="30"/>
+      <c r="B62" s="31"/>
+      <c r="C62" s="31"/>
+      <c r="D62" s="31"/>
+      <c r="E62" s="31"/>
+      <c r="F62" s="31"/>
+      <c r="G62" s="32"/>
+    </row>
+    <row r="63" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A63" s="47"/>
+      <c r="B63" s="48" t="s">
+        <v>6</v>
+      </c>
+      <c r="C63" s="49"/>
+      <c r="D63" s="65" t="s">
+        <v>10</v>
+      </c>
+      <c r="E63" s="65"/>
+      <c r="F63" s="65"/>
+      <c r="G63" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B23:B25"/>
     <mergeCell ref="E2:F2"/>
-    <mergeCell ref="A49:G49"/>
-    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="D63:F63"/>
     <mergeCell ref="B11:B13"/>
     <mergeCell ref="B14:B16"/>
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="B20:B22"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="87" fitToHeight="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="86" fitToHeight="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>